<commit_message>
Update seat data: 2026-09-14 10:45:36
</commit_message>
<xml_diff>
--- a/座位号.xlsx
+++ b/座位号.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\战略所\2026年工作\联合国创新会议\座位号程序\seatSelection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027C0C4B-8BD3-4A90-A61C-397E7B3B0E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41C86C2-7C2A-41F0-8EAB-506F5F11CBAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="84">
   <si>
     <t>编号</t>
   </si>
@@ -271,12 +271,44 @@
     <t>博士</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
+  <si>
+    <t>第一排1号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>第三排2号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>第二排15号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>第一排20号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>第一排2号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>第一排3号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>第一排4号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>第一排5号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -401,6 +433,14 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
@@ -655,7 +695,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -969,47 +1009,40 @@
       <alignment horizontal="center" vertical="center" textRotation="255"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="47">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="46">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1740,6 +1773,7 @@
     <col min="2" max="2" width="35" customWidth="1"/>
     <col min="3" max="3" width="38.125" customWidth="1"/>
     <col min="4" max="4" width="26.375" customWidth="1"/>
+    <col min="5" max="5" width="15.75" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:5">
@@ -1770,8 +1804,8 @@
       <c r="D3" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="43">
-        <v>1</v>
+      <c r="E3" s="97" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5">
@@ -1787,8 +1821,8 @@
       <c r="D4" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="43">
-        <v>2</v>
+      <c r="E4" s="97" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5">
@@ -1804,8 +1838,8 @@
       <c r="D5" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="43">
-        <v>3</v>
+      <c r="E5" s="97" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="27">
@@ -1821,8 +1855,8 @@
       <c r="D6" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="43">
-        <v>4</v>
+      <c r="E6" s="97" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16.5">
@@ -1838,62 +1872,63 @@
       <c r="D7" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="43">
-        <v>5</v>
+      <c r="E7" s="97" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5">
       <c r="A8" s="43">
         <v>6</v>
       </c>
-      <c r="B8" s="95" t="s">
+      <c r="B8" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="91" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="97" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5">
+      <c r="A9" s="43">
+        <v>7</v>
+      </c>
+      <c r="B9" s="90" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="91" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="91" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="97" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5">
+      <c r="A10" s="43">
+        <v>8</v>
+      </c>
+      <c r="B10" s="90" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="96" t="s">
+      <c r="C10" s="91" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="96" t="s">
+      <c r="D10" s="91" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="43">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="16.5">
-      <c r="A9" s="43"/>
-      <c r="B9" s="95" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" s="96" t="s">
-        <v>68</v>
-      </c>
-      <c r="D9" s="96" t="s">
-        <v>72</v>
-      </c>
-      <c r="E9" s="43">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="16.5">
-      <c r="A10" s="43"/>
-      <c r="B10" s="95" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" s="96" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="96" t="s">
-        <v>75</v>
-      </c>
-      <c r="E10" s="43">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="16.5">
+      <c r="E10" s="97" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" s="43"/>
-      <c r="B11" s="44"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
       <c r="E11" s="43"/>
     </row>
     <row r="12" spans="1:5" ht="16.5">
@@ -3382,9 +3417,6 @@
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
-  <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="46" priority="44"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B21">
     <cfRule type="duplicateValues" dxfId="45" priority="15"/>
   </conditionalFormatting>
@@ -3445,83 +3477,83 @@
   <conditionalFormatting sqref="B221:B223">
     <cfRule type="duplicateValues" dxfId="26" priority="51"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B12 B15 B6:B10">
-    <cfRule type="duplicateValues" dxfId="25" priority="46"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B16 B41:B54 B57:B63">
-    <cfRule type="duplicateValues" dxfId="24" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:B18 B22:B25 B27:B34 B37 B39 B85 B98:B99 B115 B214:B216 B218:B219">
-    <cfRule type="duplicateValues" dxfId="23" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19 B100 B188 B194 B211">
-    <cfRule type="duplicateValues" dxfId="22" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20 B101:B102 B113:B114 B171 B191:B192 B207:B208 B210">
-    <cfRule type="duplicateValues" dxfId="21" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26 B35">
-    <cfRule type="duplicateValues" dxfId="20" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B36 B93 B143">
-    <cfRule type="duplicateValues" dxfId="19" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B40 B91 B132 B137 B139:B140">
-    <cfRule type="duplicateValues" dxfId="18" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B65:B66 B73">
-    <cfRule type="duplicateValues" dxfId="17" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B67:B70 B72 B74 B76 B78 B80 B82">
-    <cfRule type="duplicateValues" dxfId="16" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B71 B79 B81 B96:B97">
-    <cfRule type="duplicateValues" dxfId="15" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B75 B178:B182 B185">
-    <cfRule type="duplicateValues" dxfId="14" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B86 B90 B122 B125">
-    <cfRule type="duplicateValues" dxfId="13" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B87 B92 B126">
-    <cfRule type="duplicateValues" dxfId="12" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B88 B109 B111 B120:B121">
-    <cfRule type="duplicateValues" dxfId="11" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B89 B220">
-    <cfRule type="duplicateValues" dxfId="10" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95 B103 B198:B199 B202:B204 B209">
-    <cfRule type="duplicateValues" dxfId="9" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B104 B106 B108 B110 B112 B177">
-    <cfRule type="duplicateValues" dxfId="8" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B105 B107">
-    <cfRule type="duplicateValues" dxfId="7" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B116:B118 B168 B172 B197">
-    <cfRule type="duplicateValues" dxfId="6" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B119 B167 B195:B196">
-    <cfRule type="duplicateValues" dxfId="5" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B124 B133 B141:B142">
-    <cfRule type="duplicateValues" dxfId="4" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B127:B128 B136 B138">
-    <cfRule type="duplicateValues" dxfId="3" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B129:B131 B193 B217">
-    <cfRule type="duplicateValues" dxfId="2" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B169:B170 B189:B190 B212:B213">
-    <cfRule type="duplicateValues" dxfId="1" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B184 B186">
-    <cfRule type="duplicateValues" dxfId="0" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="34"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15 B12 B6:B10">
+    <cfRule type="duplicateValues" dxfId="0" priority="53"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -3548,72 +3580,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:51" ht="32.1" customHeight="1">
-      <c r="Q1" s="90" t="s">
+      <c r="Q1" s="96" t="s">
         <v>19</v>
       </c>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
-      <c r="AE1" s="90"/>
-      <c r="AF1" s="90"/>
+      <c r="R1" s="96"/>
+      <c r="S1" s="96"/>
+      <c r="T1" s="96"/>
+      <c r="U1" s="96"/>
+      <c r="V1" s="96"/>
+      <c r="W1" s="96"/>
+      <c r="X1" s="96"/>
+      <c r="Y1" s="96"/>
+      <c r="Z1" s="96"/>
+      <c r="AA1" s="96"/>
+      <c r="AB1" s="96"/>
+      <c r="AC1" s="96"/>
+      <c r="AD1" s="96"/>
+      <c r="AE1" s="96"/>
+      <c r="AF1" s="96"/>
     </row>
     <row r="2" spans="1:51">
-      <c r="A2" s="91" t="s">
+      <c r="A2" s="92" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
-      <c r="N2" s="92"/>
-      <c r="O2" s="92"/>
-      <c r="P2" s="92"/>
-      <c r="Q2" s="92"/>
-      <c r="R2" s="92"/>
-      <c r="S2" s="92"/>
-      <c r="T2" s="92"/>
-      <c r="U2" s="92"/>
-      <c r="V2" s="92"/>
-      <c r="W2" s="92"/>
-      <c r="X2" s="92"/>
-      <c r="Y2" s="92"/>
-      <c r="Z2" s="92"/>
-      <c r="AA2" s="92"/>
-      <c r="AB2" s="92"/>
-      <c r="AC2" s="92"/>
-      <c r="AD2" s="92"/>
-      <c r="AE2" s="92"/>
-      <c r="AF2" s="92"/>
-      <c r="AG2" s="92"/>
-      <c r="AH2" s="92"/>
-      <c r="AI2" s="92"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="95"/>
+      <c r="Q2" s="95"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="95"/>
+      <c r="T2" s="95"/>
+      <c r="U2" s="95"/>
+      <c r="V2" s="95"/>
+      <c r="W2" s="95"/>
+      <c r="X2" s="95"/>
+      <c r="Y2" s="95"/>
+      <c r="Z2" s="95"/>
+      <c r="AA2" s="95"/>
+      <c r="AB2" s="95"/>
+      <c r="AC2" s="95"/>
+      <c r="AD2" s="95"/>
+      <c r="AE2" s="95"/>
+      <c r="AF2" s="95"/>
+      <c r="AG2" s="95"/>
+      <c r="AH2" s="95"/>
+      <c r="AI2" s="95"/>
     </row>
     <row r="3" spans="1:51">
       <c r="A3" s="2"/>
-      <c r="B3" s="91" t="s">
+      <c r="B3" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="91"/>
-      <c r="D3" s="91"/>
-      <c r="E3" s="91"/>
-      <c r="F3" s="91"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="92"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -3622,24 +3654,24 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
-      <c r="P3" s="92"/>
-      <c r="Q3" s="92"/>
-      <c r="R3" s="92"/>
-      <c r="S3" s="92"/>
-      <c r="T3" s="92"/>
-      <c r="U3" s="92"/>
-      <c r="V3" s="92"/>
-      <c r="W3" s="92"/>
-      <c r="X3" s="92"/>
-      <c r="Y3" s="92"/>
-      <c r="Z3" s="92"/>
-      <c r="AA3" s="92"/>
-      <c r="AB3" s="92"/>
-      <c r="AC3" s="92"/>
-      <c r="AD3" s="92"/>
-      <c r="AE3" s="92"/>
-      <c r="AF3" s="92"/>
-      <c r="AG3" s="92"/>
+      <c r="P3" s="95"/>
+      <c r="Q3" s="95"/>
+      <c r="R3" s="95"/>
+      <c r="S3" s="95"/>
+      <c r="T3" s="95"/>
+      <c r="U3" s="95"/>
+      <c r="V3" s="95"/>
+      <c r="W3" s="95"/>
+      <c r="X3" s="95"/>
+      <c r="Y3" s="95"/>
+      <c r="Z3" s="95"/>
+      <c r="AA3" s="95"/>
+      <c r="AB3" s="95"/>
+      <c r="AC3" s="95"/>
+      <c r="AD3" s="95"/>
+      <c r="AE3" s="95"/>
+      <c r="AF3" s="95"/>
+      <c r="AG3" s="95"/>
     </row>
     <row r="4" spans="1:51" ht="18.75">
       <c r="H4" s="3"/>
@@ -3651,34 +3683,34 @@
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="93" t="s">
+      <c r="Q4" s="94" t="s">
         <v>22</v>
       </c>
-      <c r="R4" s="92"/>
-      <c r="S4" s="92"/>
-      <c r="T4" s="92"/>
-      <c r="U4" s="92"/>
-      <c r="V4" s="92"/>
-      <c r="W4" s="92"/>
-      <c r="X4" s="92"/>
-      <c r="Y4" s="92"/>
-      <c r="Z4" s="92"/>
-      <c r="AA4" s="92"/>
-      <c r="AB4" s="92"/>
-      <c r="AC4" s="92"/>
-      <c r="AD4" s="92"/>
-      <c r="AE4" s="92"/>
-      <c r="AF4" s="92"/>
+      <c r="R4" s="95"/>
+      <c r="S4" s="95"/>
+      <c r="T4" s="95"/>
+      <c r="U4" s="95"/>
+      <c r="V4" s="95"/>
+      <c r="W4" s="95"/>
+      <c r="X4" s="95"/>
+      <c r="Y4" s="95"/>
+      <c r="Z4" s="95"/>
+      <c r="AA4" s="95"/>
+      <c r="AB4" s="95"/>
+      <c r="AC4" s="95"/>
+      <c r="AD4" s="95"/>
+      <c r="AE4" s="95"/>
+      <c r="AF4" s="95"/>
     </row>
     <row r="5" spans="1:51">
-      <c r="A5" s="91" t="s">
+      <c r="A5" s="92" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="91"/>
-      <c r="C5" s="91"/>
-      <c r="D5" s="91"/>
-      <c r="E5" s="91"/>
-      <c r="F5" s="91"/>
+      <c r="B5" s="92"/>
+      <c r="C5" s="92"/>
+      <c r="D5" s="92"/>
+      <c r="E5" s="92"/>
+      <c r="F5" s="92"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
@@ -3688,30 +3720,30 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
-      <c r="R5" s="92"/>
-      <c r="S5" s="92"/>
-      <c r="T5" s="92"/>
-      <c r="U5" s="92"/>
-      <c r="V5" s="92"/>
-      <c r="W5" s="92"/>
-      <c r="X5" s="92"/>
-      <c r="Y5" s="92"/>
-      <c r="Z5" s="92"/>
-      <c r="AA5" s="92"/>
-      <c r="AB5" s="92"/>
-      <c r="AC5" s="92"/>
-      <c r="AD5" s="92"/>
-      <c r="AE5" s="92"/>
+      <c r="R5" s="95"/>
+      <c r="S5" s="95"/>
+      <c r="T5" s="95"/>
+      <c r="U5" s="95"/>
+      <c r="V5" s="95"/>
+      <c r="W5" s="95"/>
+      <c r="X5" s="95"/>
+      <c r="Y5" s="95"/>
+      <c r="Z5" s="95"/>
+      <c r="AA5" s="95"/>
+      <c r="AB5" s="95"/>
+      <c r="AC5" s="95"/>
+      <c r="AD5" s="95"/>
+      <c r="AE5" s="95"/>
     </row>
     <row r="6" spans="1:51">
-      <c r="A6" s="91" t="s">
+      <c r="A6" s="92" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="91"/>
-      <c r="C6" s="91"/>
-      <c r="D6" s="91"/>
-      <c r="E6" s="91"/>
-      <c r="F6" s="91"/>
+      <c r="B6" s="92"/>
+      <c r="C6" s="92"/>
+      <c r="D6" s="92"/>
+      <c r="E6" s="92"/>
+      <c r="F6" s="92"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -3721,30 +3753,30 @@
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
-      <c r="S6" s="92" t="s">
+      <c r="S6" s="95" t="s">
         <v>25</v>
       </c>
-      <c r="T6" s="92"/>
-      <c r="U6" s="92"/>
-      <c r="V6" s="92"/>
-      <c r="W6" s="92"/>
-      <c r="X6" s="92"/>
-      <c r="Y6" s="92"/>
-      <c r="Z6" s="92"/>
-      <c r="AA6" s="92"/>
-      <c r="AB6" s="92"/>
-      <c r="AC6" s="92"/>
-      <c r="AD6" s="92"/>
+      <c r="T6" s="95"/>
+      <c r="U6" s="95"/>
+      <c r="V6" s="95"/>
+      <c r="W6" s="95"/>
+      <c r="X6" s="95"/>
+      <c r="Y6" s="95"/>
+      <c r="Z6" s="95"/>
+      <c r="AA6" s="95"/>
+      <c r="AB6" s="95"/>
+      <c r="AC6" s="95"/>
+      <c r="AD6" s="95"/>
     </row>
     <row r="7" spans="1:51">
-      <c r="A7" s="91" t="s">
+      <c r="A7" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="91"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
+      <c r="B7" s="92"/>
+      <c r="C7" s="92"/>
+      <c r="D7" s="92"/>
+      <c r="E7" s="92"/>
+      <c r="F7" s="92"/>
       <c r="G7" s="1">
         <v>1</v>
       </c>
@@ -3771,14 +3803,14 @@
       <c r="AD7" s="4"/>
     </row>
     <row r="8" spans="1:51">
-      <c r="A8" s="91" t="s">
+      <c r="A8" s="92" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="91"/>
-      <c r="C8" s="91"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="91"/>
+      <c r="B8" s="92"/>
+      <c r="C8" s="92"/>
+      <c r="D8" s="92"/>
+      <c r="E8" s="92"/>
+      <c r="F8" s="92"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
@@ -3919,49 +3951,48 @@
       <c r="P15" s="11"/>
       <c r="Q15" s="11"/>
       <c r="R15" s="11"/>
-      <c r="S15" s="12" t="str">
+      <c r="S15" s="12" t="e">
         <f>_xlfn.XLOOKUP(S13,人员名单!$E:$E,人员名单!$B:$B)</f>
-        <v>刘西宁</v>
+        <v>#N/A</v>
       </c>
       <c r="T15" s="11"/>
-      <c r="U15" s="12" t="str">
+      <c r="U15" s="12" t="e">
         <f>_xlfn.XLOOKUP(U13,人员名单!$E:$E,人员名单!$B:$B)</f>
-        <v>谢  京</v>
+        <v>#N/A</v>
       </c>
       <c r="V15" s="11"/>
-      <c r="W15" s="12" t="str">
+      <c r="W15" s="12" t="e">
         <f>_xlfn.XLOOKUP(W13,人员名单!$E:$E,人员名单!$B:$B)</f>
-        <v>张永涛</v>
+        <v>#N/A</v>
       </c>
       <c r="X15" s="11"/>
-      <c r="Y15" s="12" t="str">
+      <c r="Y15" s="12" t="e">
         <f>_xlfn.XLOOKUP(Y13,人员名单!$E:$E,人员名单!$B:$B)</f>
-        <v>王祺扬</v>
+        <v>#N/A</v>
       </c>
       <c r="Z15" s="11"/>
-      <c r="AA15" s="12" t="str">
+      <c r="AA15" s="12" t="e">
         <f>_xlfn.XLOOKUP(AA13,人员名单!$E:$E,人员名单!$B:$B)</f>
-        <v>孙  键</v>
+        <v>#N/A</v>
       </c>
       <c r="AB15" s="11"/>
-      <c r="AC15" s="12" t="str">
+      <c r="AC15" s="12" t="e">
         <f>_xlfn.XLOOKUP(AC13,人员名单!$E:$E,人员名单!$B:$B)</f>
-        <v>FARID CHEMALE JUNlOR
-法里德·谢马莱·朱尼尔</v>
+        <v>#N/A</v>
       </c>
       <c r="AD15" s="11"/>
-      <c r="AE15" s="12" t="str">
+      <c r="AE15" s="12" t="e">
         <f>_xlfn.XLOOKUP(AE13,人员名单!$E:$E,人员名单!$B:$B)</f>
-        <v>唐  享</v>
+        <v>#N/A</v>
       </c>
       <c r="AF15" s="11"/>
       <c r="AG15" s="11"/>
       <c r="AH15" s="11"/>
       <c r="AI15" s="11"/>
       <c r="AJ15" s="11"/>
-      <c r="AK15" s="12" t="str">
+      <c r="AK15" s="12" t="e">
         <f>_xlfn.XLOOKUP(AK13,人员名单!$E:$E,人员名单!$B:$B)</f>
-        <v>杨  刚</v>
+        <v>#N/A</v>
       </c>
       <c r="AL15" s="11"/>
       <c r="AM15" s="12" t="e">
@@ -5057,7 +5088,7 @@
       </c>
       <c r="AW26" s="15"/>
     </row>
-    <row r="27" spans="1:51" ht="42">
+    <row r="27" spans="1:51" ht="55.5">
       <c r="A27" s="15"/>
       <c r="D27" s="20" t="e">
         <f>_xlfn.XLOOKUP(D26,人员名单!$E:$E,人员名单!$B:$B)</f>
@@ -8657,24 +8688,24 @@
       </c>
     </row>
     <row r="65" spans="5:44">
-      <c r="O65" s="94" t="s">
+      <c r="O65" s="93" t="s">
         <v>54</v>
       </c>
-      <c r="P65" s="94"/>
-      <c r="AH65" s="94" t="s">
+      <c r="P65" s="93"/>
+      <c r="AH65" s="93" t="s">
         <v>54</v>
       </c>
-      <c r="AI65" s="94"/>
+      <c r="AI65" s="93"/>
     </row>
     <row r="66" spans="5:44">
-      <c r="O66" s="94" t="s">
+      <c r="O66" s="93" t="s">
         <v>55</v>
       </c>
-      <c r="P66" s="94"/>
-      <c r="AH66" s="94" t="s">
+      <c r="P66" s="93"/>
+      <c r="AH66" s="93" t="s">
         <v>55</v>
       </c>
-      <c r="AI66" s="94"/>
+      <c r="AI66" s="93"/>
     </row>
     <row r="68" spans="5:44">
       <c r="E68" s="36"/>
@@ -8738,23 +8769,23 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="Q1:AF1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="N2:AE2"/>
+    <mergeCell ref="AF2:AI2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="P3:AG3"/>
+    <mergeCell ref="Q4:AF4"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="R5:AE5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="S6:AD6"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="O65:P65"/>
     <mergeCell ref="AH65:AI65"/>
     <mergeCell ref="O66:P66"/>
     <mergeCell ref="AH66:AI66"/>
-    <mergeCell ref="Q4:AF4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="R5:AE5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="S6:AD6"/>
-    <mergeCell ref="Q1:AF1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="N2:AE2"/>
-    <mergeCell ref="AF2:AI2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="P3:AG3"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>